<commit_message>
added simulation study for PED (item sets balanced across replications), updated codebook to include positive emotions
</commit_message>
<xml_diff>
--- a/prepared data/codebook_benchmark_data.xlsx
+++ b/prepared data/codebook_benchmark_data.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A2B5C27-5B11-45E6-AD53-566934A4ABC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B34E613-82A2-4497-90E9-50B86E4AFF82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4005" yWindow="7995" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="68">
   <si>
     <t>SERIAL</t>
   </si>
@@ -53,9 +53,6 @@
 100 = very strong</t>
   </si>
   <si>
-    <t>instruction for all emotion items (aerger1 to schuld3): Please indicate your feelings within the past hour.</t>
-  </si>
-  <si>
     <t>aerger2</t>
   </si>
   <si>
@@ -156,6 +153,81 @@
   </si>
   <si>
     <t>Note / Instruction</t>
+  </si>
+  <si>
+    <t>freude1</t>
+  </si>
+  <si>
+    <t>freude2</t>
+  </si>
+  <si>
+    <t>freude3</t>
+  </si>
+  <si>
+    <t>interesse1</t>
+  </si>
+  <si>
+    <t>interesse2</t>
+  </si>
+  <si>
+    <t>interesse3</t>
+  </si>
+  <si>
+    <t>liebe1</t>
+  </si>
+  <si>
+    <t>liebe2</t>
+  </si>
+  <si>
+    <t>liebe3</t>
+  </si>
+  <si>
+    <t>stolz1</t>
+  </si>
+  <si>
+    <t>stolz2</t>
+  </si>
+  <si>
+    <t>stolz3</t>
+  </si>
+  <si>
+    <t>instruction for all emotion items (aerger1 to stolz3): Please indicate your feelings within the past hour.</t>
+  </si>
+  <si>
+    <t>joyful</t>
+  </si>
+  <si>
+    <t>glad</t>
+  </si>
+  <si>
+    <t>happy</t>
+  </si>
+  <si>
+    <t>interested</t>
+  </si>
+  <si>
+    <t>alert</t>
+  </si>
+  <si>
+    <t>curious</t>
+  </si>
+  <si>
+    <t>love</t>
+  </si>
+  <si>
+    <t>closeness</t>
+  </si>
+  <si>
+    <t>trust</t>
+  </si>
+  <si>
+    <t>proud</t>
+  </si>
+  <si>
+    <t>confident</t>
+  </si>
+  <si>
+    <t>self-assured</t>
   </si>
 </sst>
 </file>
@@ -508,7 +580,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.28515625" customWidth="1"/>
@@ -519,7 +591,7 @@
   <sheetData>
     <row r="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -535,7 +607,7 @@
         <v>3</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -556,19 +628,19 @@
     </row>
     <row r="6" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C6" s="5"/>
     </row>
     <row r="7" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" s="8" t="s">
         <v>40</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -582,15 +654,15 @@
         <v>8</v>
       </c>
       <c r="D8" t="s">
-        <v>9</v>
+        <v>55</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
         <v>10</v>
-      </c>
-      <c r="B9" t="s">
-        <v>11</v>
       </c>
       <c r="C9" s="7" t="s">
         <v>8</v>
@@ -598,10 +670,10 @@
     </row>
     <row r="10" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" t="s">
         <v>12</v>
-      </c>
-      <c r="B10" t="s">
-        <v>13</v>
       </c>
       <c r="C10" s="7" t="s">
         <v>8</v>
@@ -609,10 +681,10 @@
     </row>
     <row r="11" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" t="s">
         <v>14</v>
-      </c>
-      <c r="B11" t="s">
-        <v>15</v>
       </c>
       <c r="C11" s="7" t="s">
         <v>8</v>
@@ -620,10 +692,10 @@
     </row>
     <row r="12" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B12" t="s">
         <v>16</v>
-      </c>
-      <c r="B12" t="s">
-        <v>17</v>
       </c>
       <c r="C12" s="7" t="s">
         <v>8</v>
@@ -631,10 +703,10 @@
     </row>
     <row r="13" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13" t="s">
         <v>18</v>
-      </c>
-      <c r="B13" t="s">
-        <v>19</v>
       </c>
       <c r="C13" s="7" t="s">
         <v>8</v>
@@ -642,10 +714,10 @@
     </row>
     <row r="14" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" t="s">
         <v>20</v>
-      </c>
-      <c r="B14" t="s">
-        <v>21</v>
       </c>
       <c r="C14" s="7" t="s">
         <v>8</v>
@@ -653,10 +725,10 @@
     </row>
     <row r="15" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>21</v>
+      </c>
+      <c r="B15" t="s">
         <v>22</v>
-      </c>
-      <c r="B15" t="s">
-        <v>23</v>
       </c>
       <c r="C15" s="7" t="s">
         <v>8</v>
@@ -664,10 +736,10 @@
     </row>
     <row r="16" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>23</v>
+      </c>
+      <c r="B16" t="s">
         <v>24</v>
-      </c>
-      <c r="B16" t="s">
-        <v>25</v>
       </c>
       <c r="C16" s="7" t="s">
         <v>8</v>
@@ -675,10 +747,10 @@
     </row>
     <row r="17" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>25</v>
+      </c>
+      <c r="B17" t="s">
         <v>26</v>
-      </c>
-      <c r="B17" t="s">
-        <v>27</v>
       </c>
       <c r="C17" s="7" t="s">
         <v>8</v>
@@ -686,10 +758,10 @@
     </row>
     <row r="18" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18" t="s">
         <v>28</v>
-      </c>
-      <c r="B18" t="s">
-        <v>29</v>
       </c>
       <c r="C18" s="7" t="s">
         <v>8</v>
@@ -697,10 +769,10 @@
     </row>
     <row r="19" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>29</v>
+      </c>
+      <c r="B19" t="s">
         <v>30</v>
-      </c>
-      <c r="B19" t="s">
-        <v>31</v>
       </c>
       <c r="C19" s="7" t="s">
         <v>8</v>
@@ -708,10 +780,10 @@
     </row>
     <row r="20" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>31</v>
+      </c>
+      <c r="B20" t="s">
         <v>32</v>
-      </c>
-      <c r="B20" t="s">
-        <v>33</v>
       </c>
       <c r="C20" s="7" t="s">
         <v>8</v>
@@ -719,10 +791,10 @@
     </row>
     <row r="21" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>33</v>
+      </c>
+      <c r="B21" t="s">
         <v>34</v>
-      </c>
-      <c r="B21" t="s">
-        <v>35</v>
       </c>
       <c r="C21" s="7" t="s">
         <v>8</v>
@@ -730,17 +802,149 @@
     </row>
     <row r="22" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>35</v>
+      </c>
+      <c r="B22" t="s">
         <v>36</v>
       </c>
-      <c r="B22" t="s">
-        <v>37</v>
-      </c>
       <c r="C22" s="7" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C23" s="8"/>
+    <row r="23" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>43</v>
+      </c>
+      <c r="B23" t="s">
+        <v>56</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24" t="s">
+        <v>57</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25" t="s">
+        <v>58</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26" t="s">
+        <v>59</v>
+      </c>
+      <c r="C26" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27" t="s">
+        <v>60</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>48</v>
+      </c>
+      <c r="B28" t="s">
+        <v>61</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>49</v>
+      </c>
+      <c r="B29" t="s">
+        <v>62</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>50</v>
+      </c>
+      <c r="B30" t="s">
+        <v>63</v>
+      </c>
+      <c r="C30" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>51</v>
+      </c>
+      <c r="B31" t="s">
+        <v>64</v>
+      </c>
+      <c r="C31" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>52</v>
+      </c>
+      <c r="B32" t="s">
+        <v>65</v>
+      </c>
+      <c r="C32" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>53</v>
+      </c>
+      <c r="B33" t="s">
+        <v>66</v>
+      </c>
+      <c r="C33" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>54</v>
+      </c>
+      <c r="B34" t="s">
+        <v>67</v>
+      </c>
+      <c r="C34" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C35" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>